<commit_message>
update map of scripts
</commit_message>
<xml_diff>
--- a/Guide to Project.xlsx
+++ b/Guide to Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jball\Documents\local-git\KRSP_exploring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9ABFEA0-B5B7-42CF-9F6A-24A8788C7A4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E6E05CD-40E5-4819-B1E4-CA24D6A9C879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8DBE1842-90D7-491B-B4CD-F8D8B6831160}"/>
+    <workbookView xWindow="3516" yWindow="216" windowWidth="18660" windowHeight="11892" activeTab="1" xr2:uid="{8DBE1842-90D7-491B-B4CD-F8D8B6831160}"/>
   </bookViews>
   <sheets>
     <sheet name="Steps and Sample Sizes" sheetId="1" r:id="rId1"/>
@@ -1710,16 +1710,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>188595</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>17145</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>325755</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>78105</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>217170</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>354330</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:rowOff>26670</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1734,8 +1734,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5065395" y="5265420"/>
-          <a:ext cx="1247775" cy="493395"/>
+          <a:off x="4592955" y="5198745"/>
+          <a:ext cx="1247775" cy="497205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1774,78 +1774,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>331470</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
+      <xdr:colOff>251459</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>108585</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>344805</xdr:colOff>
+      <xdr:colOff>390524</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="111" name="Rectangle 110">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3CB1DFA1-25AE-46CB-8A28-6B7C20DF47AA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6427470" y="5250180"/>
-          <a:ext cx="1232535" cy="501015"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>10-lm_figures</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>449579</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>588644</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1860,8 +1797,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7764779" y="5257800"/>
-          <a:ext cx="1358265" cy="497205"/>
+          <a:off x="6347459" y="5229225"/>
+          <a:ext cx="1358265" cy="501015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1890,7 +1827,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>11_bayesian_models</a:t>
+            <a:t>10_bayesian_models</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1899,16 +1836,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>592455</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>28574</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1905</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1923,8 +1860,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3030855" y="6364605"/>
-          <a:ext cx="1238250" cy="476250"/>
+          <a:off x="3076574" y="9669780"/>
+          <a:ext cx="1777366" cy="480060"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1953,7 +1890,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>14-figure_density</a:t>
+            <a:t>15-density_method_figure</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1962,16 +1899,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>179069</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>232409</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>459104</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1986,8 +1923,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6884669" y="6301740"/>
-          <a:ext cx="1499235" cy="485775"/>
+          <a:off x="5109209" y="6435090"/>
+          <a:ext cx="1116331" cy="491490"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2016,7 +1953,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>12-bayesian_results</a:t>
+            <a:t>11-ellipse_figure</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2025,16 +1962,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>556258</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>213358</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>461009</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>93345</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2049,8 +1986,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8481058" y="6301740"/>
-          <a:ext cx="1733551" cy="487680"/>
+          <a:off x="5090158" y="7349490"/>
+          <a:ext cx="2110742" cy="493395"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2079,8 +2016,13 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>13-bayesian_predictions</a:t>
+            <a:t>12-covariance_correlation</a:t>
           </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>_figure</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -2088,16 +2030,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>201930</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>340043</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>49530</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>321945</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>20955</xdr:rowOff>
+      <xdr:colOff>325755</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>78105</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2115,8 +2057,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="5688330" y="4754880"/>
-          <a:ext cx="1339215" cy="514350"/>
+          <a:off x="5216843" y="4802505"/>
+          <a:ext cx="1814512" cy="396240"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2145,71 +2087,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>321945</xdr:colOff>
+      <xdr:colOff>320992</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>49530</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>337185</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>1905</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="119" name="Straight Arrow Connector 118">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9B47B85-7682-16BA-7139-DC724FC9D146}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="60" idx="2"/>
-          <a:endCxn id="111" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7027545" y="4754880"/>
-          <a:ext cx="15240" cy="495300"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>321945</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>49530</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>520064</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>11430</xdr:rowOff>
+      <xdr:colOff>325755</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>108585</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2226,9 +2112,9 @@
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7027545" y="4754880"/>
-          <a:ext cx="1417319" cy="504825"/>
+        <a:xfrm flipH="1">
+          <a:off x="7026592" y="4802505"/>
+          <a:ext cx="4763" cy="426720"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2256,16 +2142,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>317182</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>520064</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>320992</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2283,8 +2169,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="7632382" y="5753100"/>
-          <a:ext cx="812482" cy="548640"/>
+          <a:off x="5667375" y="5730240"/>
+          <a:ext cx="1359217" cy="704850"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2312,16 +2198,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>520064</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>49529</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>201929</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>320992</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2338,9 +2224,9 @@
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8444864" y="5753100"/>
-          <a:ext cx="901065" cy="548640"/>
+        <a:xfrm flipH="1">
+          <a:off x="6145529" y="5730240"/>
+          <a:ext cx="881063" cy="1619250"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2368,16 +2254,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>307658</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>29527</xdr:rowOff>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>443865</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>28574</xdr:rowOff>
+      <xdr:colOff>445771</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2395,10 +2281,248 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000" flipV="1">
-          <a:off x="3648075" y="2020252"/>
-          <a:ext cx="453390" cy="4342447"/>
+          <a:off x="3965258" y="2042160"/>
+          <a:ext cx="138113" cy="7627620"/>
         </a:xfrm>
         <a:prstGeom prst="bentConnector2">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>7618</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>118110</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>289560</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>62865</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="47" name="Rectangle 46">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DC21E9C-1AB4-4E8F-9CFA-A46A12876EE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6713218" y="8164830"/>
+          <a:ext cx="2110742" cy="493395"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>13-separate_linear_predictions</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>320992</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>453389</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>118110</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="51" name="Straight Arrow Connector 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8593CEE8-8C3A-4692-8680-2325A4BC0B97}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="112" idx="2"/>
+          <a:endCxn id="47" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7026592" y="5730240"/>
+          <a:ext cx="741997" cy="2434590"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>45718</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>327660</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="Rectangle 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF2FC272-3372-487F-A422-C45D13CEF289}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8580118" y="8812530"/>
+          <a:ext cx="2110742" cy="493395"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>14-posterior_distributions</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>320992</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>491489</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="77" name="Straight Arrow Connector 76">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{243C068F-45A6-40C5-8560-6747DD5747C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="112" idx="2"/>
+          <a:endCxn id="57" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7026592" y="5730240"/>
+          <a:ext cx="2608897" cy="3082290"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
           <a:avLst/>
         </a:prstGeom>
         <a:ln>

</xml_diff>

<commit_message>
update names on map
</commit_message>
<xml_diff>
--- a/Guide to Project.xlsx
+++ b/Guide to Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jball\Documents\local-git\KRSP_exploring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E6E05CD-40E5-4819-B1E4-CA24D6A9C879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D803EA05-46B9-4A94-932D-824BC1BCF6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3516" yWindow="216" windowWidth="18660" windowHeight="11892" activeTab="1" xr2:uid="{8DBE1842-90D7-491B-B4CD-F8D8B6831160}"/>
+    <workbookView xWindow="2820" yWindow="312" windowWidth="18660" windowHeight="11892" activeTab="1" xr2:uid="{8DBE1842-90D7-491B-B4CD-F8D8B6831160}"/>
   </bookViews>
   <sheets>
     <sheet name="Steps and Sample Sizes" sheetId="1" r:id="rId1"/>
@@ -411,15 +411,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>445770</xdr:colOff>
+      <xdr:colOff>430530</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:rowOff>148590</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>169545</xdr:colOff>
+      <xdr:colOff>154305</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>102870</xdr:rowOff>
+      <xdr:rowOff>110490</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -434,8 +434,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4103370" y="1769745"/>
-          <a:ext cx="942975" cy="504825"/>
+          <a:off x="4088130" y="1794510"/>
+          <a:ext cx="942975" cy="510540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -920,15 +920,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>308610</xdr:colOff>
+      <xdr:colOff>292418</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>56198</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>139065</xdr:rowOff>
+      <xdr:rowOff>148590</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -946,8 +946,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="4575810" y="990600"/>
-          <a:ext cx="2795588" cy="777240"/>
+          <a:off x="4559618" y="998220"/>
+          <a:ext cx="2811780" cy="796290"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -976,15 +976,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>297180</xdr:colOff>
+      <xdr:colOff>292418</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>100965</xdr:rowOff>
+      <xdr:rowOff>110490</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>308610</xdr:colOff>
+      <xdr:colOff>294323</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1001,9 +1001,9 @@
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="4564380" y="2272665"/>
-          <a:ext cx="11430" cy="314325"/>
+        <a:xfrm>
+          <a:off x="4559618" y="2305050"/>
+          <a:ext cx="1905" cy="312420"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1256,15 +1256,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>308610</xdr:colOff>
+      <xdr:colOff>292418</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>376238</xdr:colOff>
+      <xdr:colOff>377190</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>139065</xdr:rowOff>
+      <xdr:rowOff>148590</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1282,8 +1282,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="4575810" y="990600"/>
-          <a:ext cx="677228" cy="777240"/>
+          <a:off x="4559618" y="998220"/>
+          <a:ext cx="694372" cy="796290"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1710,16 +1710,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>325755</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>78105</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>354330</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>26670</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>539115</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>93345</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>567690</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>41910</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1734,7 +1734,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4592955" y="5198745"/>
+          <a:off x="4196715" y="4848225"/>
           <a:ext cx="1247775" cy="497205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1836,16 +1836,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>28574</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>59054</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>586740</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>106680</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1860,7 +1860,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3076574" y="9669780"/>
+          <a:off x="2497454" y="9136380"/>
           <a:ext cx="1777366" cy="480060"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1890,7 +1890,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>15-density_method_figure</a:t>
+            <a:t>16-density_method_figure</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1899,16 +1899,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>232409</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>129540</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>323849</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>72390</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1923,7 +1923,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5109209" y="6435090"/>
+          <a:off x="4591049" y="6107430"/>
           <a:ext cx="1116331" cy="491490"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1962,16 +1962,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>213358</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>419098</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>78105</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1986,7 +1986,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5090158" y="7349490"/>
+          <a:off x="4686298" y="6717030"/>
           <a:ext cx="2110742" cy="493395"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2030,62 +2030,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>340043</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>325755</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>78105</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="117" name="Straight Arrow Connector 116">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C27E0F97-F696-21DA-8B59-B453894F6135}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="60" idx="2"/>
-          <a:endCxn id="110" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="5216843" y="4802505"/>
-          <a:ext cx="1814512" cy="396240"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>320992</xdr:colOff>
       <xdr:row>26</xdr:row>
@@ -2142,16 +2086,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>272415</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>320992</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>72390</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2169,8 +2113,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="5667375" y="5730240"/>
-          <a:ext cx="1359217" cy="704850"/>
+          <a:off x="5149215" y="5730240"/>
+          <a:ext cx="1877377" cy="377190"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2198,16 +2142,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>49529</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>255269</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>320992</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2225,8 +2169,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="6145529" y="5730240"/>
-          <a:ext cx="881063" cy="1619250"/>
+          <a:off x="5741669" y="5730240"/>
+          <a:ext cx="1284923" cy="986790"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2254,16 +2198,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>338138</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>307658</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>445771</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:colOff>430531</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2281,8 +2225,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm rot="10800000" flipV="1">
-          <a:off x="3965258" y="2042160"/>
-          <a:ext cx="138113" cy="7627620"/>
+          <a:off x="3386138" y="2049780"/>
+          <a:ext cx="701993" cy="7086600"/>
         </a:xfrm>
         <a:prstGeom prst="bentConnector2">
           <a:avLst/>
@@ -2310,16 +2254,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>7618</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>118110</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>289560</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>62865</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>495298</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>49530</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>177165</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2334,7 +2278,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6713218" y="8164830"/>
+          <a:off x="5981698" y="7364730"/>
           <a:ext cx="2110742" cy="493395"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2379,10 +2323,10 @@
       <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>453389</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>118110</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>331469</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>49530</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2401,7 +2345,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7026592" y="5730240"/>
-          <a:ext cx="741997" cy="2434590"/>
+          <a:ext cx="10477" cy="1634490"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2429,16 +2373,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>45718</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>327660</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>243838</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>525780</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>24765</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2453,7 +2397,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8580118" y="8812530"/>
+          <a:off x="7559038" y="7943850"/>
           <a:ext cx="2110742" cy="493395"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2498,10 +2442,10 @@
       <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>491489</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>34290</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>80009</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2520,9 +2464,184 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7026592" y="5730240"/>
-          <a:ext cx="2608897" cy="3082290"/>
+          <a:ext cx="1587817" cy="2213610"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>449578</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>125730</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>121920</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>70485</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="Rectangle 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85360E0B-3C4C-4D14-ADD7-4833A1A9EF19}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9593578" y="8538210"/>
+          <a:ext cx="2110742" cy="493395"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>15-bayesian_model_tables</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>320992</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>285749</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>125730</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="25" name="Straight Arrow Connector 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87E58BB1-F2E4-4E31-B1D7-C163AC2E5790}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="112" idx="2"/>
+          <a:endCxn id="18" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7026592" y="5730240"/>
+          <a:ext cx="3622357" cy="2807970"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>553403</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>31433</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>135255</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>93345</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="36" name="Connector: Elbow 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E500FFD-9C07-B958-EF15-57BD149D32F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="60" idx="1"/>
+          <a:endCxn id="110" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000" flipV="1">
+          <a:off x="4820603" y="4603433"/>
+          <a:ext cx="1410652" cy="244792"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector2">
           <a:avLst/>
         </a:prstGeom>
         <a:ln>

</xml_diff>

<commit_message>
rename scripts in map
</commit_message>
<xml_diff>
--- a/Guide to Project.xlsx
+++ b/Guide to Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jball\Documents\local-git\KRSP_exploring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D803EA05-46B9-4A94-932D-824BC1BCF6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0877818F-67CE-4EF9-BF3A-D177FEBB266F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2820" yWindow="312" windowWidth="18660" windowHeight="11892" activeTab="1" xr2:uid="{8DBE1842-90D7-491B-B4CD-F8D8B6831160}"/>
+    <workbookView xWindow="2820" yWindow="312" windowWidth="18660" windowHeight="11892" xr2:uid="{8DBE1842-90D7-491B-B4CD-F8D8B6831160}"/>
   </bookViews>
   <sheets>
     <sheet name="Steps and Sample Sizes" sheetId="1" r:id="rId1"/>
@@ -1421,7 +1421,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>08-final_merge</a:t>
+            <a:t>07-final_merge</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1764,7 +1764,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>09-summary_fig</a:t>
+            <a:t>08-summary_fig</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1827,7 +1827,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>10_bayesian_models</a:t>
+            <a:t>09_bayesian_models</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1890,7 +1890,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>16-density_method_figure</a:t>
+            <a:t>15-density_method_figure</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1953,7 +1953,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>11-ellipse_figure</a:t>
+            <a:t>10-ellipse_figure</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2016,7 +2016,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>12-covariance_correlation</a:t>
+            <a:t>11-covariance_correlation</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>
@@ -2308,7 +2308,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>13-separate_linear_predictions</a:t>
+            <a:t>12-separate_linear_predictions</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2427,7 +2427,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>14-posterior_distributions</a:t>
+            <a:t>13-posterior_distributions</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2546,7 +2546,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>15-bayesian_model_tables</a:t>
+            <a:t>14-bayesian_model_tables</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>

</xml_diff>